<commit_message>
Automatsko ažuriranje artikli.xlsx iz POS sistema
</commit_message>
<xml_diff>
--- a/artikli.xlsx
+++ b/artikli.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5099"/>
+  <dimension ref="A1:D5149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2703,7 +2703,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="128">
@@ -3225,7 +3225,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>0.72</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="157">
@@ -4377,7 +4377,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>0.8</v>
+        <v>0.7000000000000001</v>
       </c>
     </row>
     <row r="221">
@@ -4539,7 +4539,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="230">
@@ -4899,7 +4899,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="250">
@@ -8531,11 +8531,11 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>TRAVARICA 0,10 L</t>
+          <t>TRAVARICA 0,10L</t>
         </is>
       </c>
       <c r="D451" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="452">
@@ -9413,11 +9413,11 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>KLAS MILK ROLLS 300 G</t>
+          <t>KLAS MILK ROLLS 300G</t>
         </is>
       </c>
       <c r="D500" t="n">
-        <v>4.2</v>
+        <v>4.100000000000001</v>
       </c>
     </row>
     <row r="501">
@@ -9597,7 +9597,7 @@
         </is>
       </c>
       <c r="D510" t="n">
-        <v>4.899999999999999</v>
+        <v>5.199999999999999</v>
       </c>
     </row>
     <row r="511">
@@ -11793,7 +11793,7 @@
         </is>
       </c>
       <c r="D632" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="633">
@@ -12185,11 +12185,11 @@
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>PEZ IGRACKA 17 G</t>
+          <t>PEZ IGRACKA 17G</t>
         </is>
       </c>
       <c r="D654" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="655">
@@ -15281,11 +15281,11 @@
       </c>
       <c r="C826" t="inlineStr">
         <is>
-          <t>SODA BIKARBONA 250 G</t>
+          <t>SODA BIKARBONA 250G</t>
         </is>
       </c>
       <c r="D826" t="n">
-        <v>2.7</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="827">
@@ -16577,7 +16577,7 @@
       </c>
       <c r="C898" t="inlineStr">
         <is>
-          <t>VOCNA KASA JABUKA KRUSKA I BANANA 100 G</t>
+          <t>VOCNA KASA JAB&amp;KRU&amp;BAN 100G</t>
         </is>
       </c>
       <c r="D898" t="n">
@@ -17013,7 +17013,7 @@
         </is>
       </c>
       <c r="D922" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="923">
@@ -17927,11 +17927,11 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>DOVE REFRESHING</t>
+          <t>DOVE GO FRESH 90G</t>
         </is>
       </c>
       <c r="D973" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="974">
@@ -22499,11 +22499,11 @@
       </c>
       <c r="C1227" t="inlineStr">
         <is>
-          <t>CIK CAK VATA 50 G</t>
+          <t>SANITETSKA VATA CIK-CAK 50G</t>
         </is>
       </c>
       <c r="D1227" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="1228">
@@ -22517,11 +22517,11 @@
       </c>
       <c r="C1228" t="inlineStr">
         <is>
-          <t>CIK CAK VATA 100 G</t>
+          <t>SANITETSKA VATA CIK-CAK 100G</t>
         </is>
       </c>
       <c r="D1228" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1229">
@@ -23313,7 +23313,7 @@
         </is>
       </c>
       <c r="D1272" t="n">
-        <v>14.6</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="1273">
@@ -24771,7 +24771,7 @@
         </is>
       </c>
       <c r="D1353" t="n">
-        <v>3.78</v>
+        <v>3.73</v>
       </c>
     </row>
     <row r="1354">
@@ -25833,7 +25833,7 @@
         </is>
       </c>
       <c r="D1412" t="n">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="1413">
@@ -25901,7 +25901,7 @@
       </c>
       <c r="C1416" t="inlineStr">
         <is>
-          <t>MOJA KRAVICA COKOLADNO MLIJEKO 1 L</t>
+          <t>MOJA KRAVICA COKOLADNO MLIJEKO 1L</t>
         </is>
       </c>
       <c r="D1416" t="n">
@@ -25941,7 +25941,7 @@
         </is>
       </c>
       <c r="D1418" t="n">
-        <v>1.23</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="1419">
@@ -25959,7 +25959,7 @@
         </is>
       </c>
       <c r="D1419" t="n">
-        <v>1.01</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="1420">
@@ -26283,7 +26283,7 @@
         </is>
       </c>
       <c r="D1437" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="1438">
@@ -29973,7 +29973,7 @@
         </is>
       </c>
       <c r="D1642" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="1643">
@@ -31197,7 +31197,7 @@
         </is>
       </c>
       <c r="D1710" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="1711">
@@ -31233,7 +31233,7 @@
         </is>
       </c>
       <c r="D1712" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="1713">
@@ -31395,7 +31395,7 @@
         </is>
       </c>
       <c r="D1721" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="1722">
@@ -32295,7 +32295,7 @@
         </is>
       </c>
       <c r="D1771" t="n">
-        <v>1.63</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="1772">
@@ -32313,7 +32313,7 @@
         </is>
       </c>
       <c r="D1772" t="n">
-        <v>1.62</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="1773">
@@ -32331,7 +32331,7 @@
         </is>
       </c>
       <c r="D1773" t="n">
-        <v>1.48</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="1774">
@@ -32385,7 +32385,7 @@
         </is>
       </c>
       <c r="D1776" t="n">
-        <v>1.62</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="1777">
@@ -32673,7 +32673,7 @@
         </is>
       </c>
       <c r="D1792" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1793">
@@ -32781,7 +32781,7 @@
         </is>
       </c>
       <c r="D1798" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="1799">
@@ -33231,7 +33231,7 @@
         </is>
       </c>
       <c r="D1823" t="n">
-        <v>3.8</v>
+        <v>4.399999999999999</v>
       </c>
     </row>
     <row r="1824">
@@ -34275,7 +34275,7 @@
         </is>
       </c>
       <c r="D1881" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="1882">
@@ -34311,7 +34311,7 @@
         </is>
       </c>
       <c r="D1883" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="1884">
@@ -34779,7 +34779,7 @@
         </is>
       </c>
       <c r="D1909" t="n">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="1910">
@@ -36939,7 +36939,7 @@
         </is>
       </c>
       <c r="D2029" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="2030">
@@ -36975,7 +36975,7 @@
         </is>
       </c>
       <c r="D2031" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="2032">
@@ -37191,7 +37191,7 @@
         </is>
       </c>
       <c r="D2043" t="n">
-        <v>9</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="2044">
@@ -37227,7 +37227,7 @@
         </is>
       </c>
       <c r="D2045" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="2046">
@@ -37353,7 +37353,7 @@
         </is>
       </c>
       <c r="D2052" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="2053">
@@ -41097,7 +41097,7 @@
         </is>
       </c>
       <c r="D2260" t="n">
-        <v>6.3</v>
+        <v>6.399999999999999</v>
       </c>
     </row>
     <row r="2261">
@@ -42231,7 +42231,7 @@
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="2324">
@@ -46047,7 +46047,7 @@
         </is>
       </c>
       <c r="D2535" t="n">
-        <v>1.8</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="2536">
@@ -47145,7 +47145,7 @@
         </is>
       </c>
       <c r="D2596" t="n">
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="2597">
@@ -47883,7 +47883,7 @@
         </is>
       </c>
       <c r="D2637" t="n">
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="2638">
@@ -47901,7 +47901,7 @@
         </is>
       </c>
       <c r="D2638" t="n">
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="2639">
@@ -51663,7 +51663,7 @@
         </is>
       </c>
       <c r="D2847" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="2848">
@@ -51897,7 +51897,7 @@
         </is>
       </c>
       <c r="D2860" t="n">
-        <v>4.8</v>
+        <v>5.899999999999999</v>
       </c>
     </row>
     <row r="2861">
@@ -52149,7 +52149,7 @@
         </is>
       </c>
       <c r="D2874" t="n">
-        <v>0.8</v>
+        <v>0.7000000000000001</v>
       </c>
     </row>
     <row r="2875">
@@ -54219,7 +54219,7 @@
         </is>
       </c>
       <c r="D2989" t="n">
-        <v>0.8</v>
+        <v>0.7000000000000001</v>
       </c>
     </row>
     <row r="2990">
@@ -56667,7 +56667,7 @@
         </is>
       </c>
       <c r="D3125" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="3126">
@@ -58341,7 +58341,7 @@
         </is>
       </c>
       <c r="D3218" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="3219">
@@ -58485,7 +58485,7 @@
         </is>
       </c>
       <c r="D3226" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3227">
@@ -58989,7 +58989,7 @@
         </is>
       </c>
       <c r="D3254" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3255">
@@ -59223,7 +59223,7 @@
         </is>
       </c>
       <c r="D3267" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="3268">
@@ -65343,7 +65343,7 @@
         </is>
       </c>
       <c r="D3607" t="n">
-        <v>7.699999999999999</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="3608">
@@ -65739,7 +65739,7 @@
         </is>
       </c>
       <c r="D3629" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="3630">
@@ -66549,7 +66549,7 @@
         </is>
       </c>
       <c r="D3674" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="3675">
@@ -68309,11 +68309,11 @@
       </c>
       <c r="C3772" t="inlineStr">
         <is>
-          <t>CAJ KAMILICA 20G</t>
+          <t>PODRAVKA CAJ KAMILICA 20G</t>
         </is>
       </c>
       <c r="D3772" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="3773">
@@ -68885,7 +68885,7 @@
       </c>
       <c r="C3804" t="inlineStr">
         <is>
-          <t>VIDAL WILD STRAWBERRIES 90G</t>
+          <t>VIDAL DIVLJA JAGODA 90G</t>
         </is>
       </c>
       <c r="D3804" t="n">
@@ -70343,7 +70343,7 @@
       </c>
       <c r="C3885" t="inlineStr">
         <is>
-          <t>VIDAL MORSKI PAS 90G GUMENE</t>
+          <t>VIDAL MORSKI PAS 90G</t>
         </is>
       </c>
       <c r="D3885" t="n">
@@ -70937,7 +70937,7 @@
       </c>
       <c r="C3918" t="inlineStr">
         <is>
-          <t>VIDAL SOUR COLA BOTTLES 90G</t>
+          <t>VIDAL KISELE COLA FLASICE 90G</t>
         </is>
       </c>
       <c r="D3918" t="n">
@@ -71211,7 +71211,7 @@
         </is>
       </c>
       <c r="D3933" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="3934">
@@ -75891,7 +75891,7 @@
         </is>
       </c>
       <c r="D4193" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="4194">
@@ -85683,7 +85683,7 @@
         </is>
       </c>
       <c r="D4737" t="n">
-        <v>1.16</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="4738">
@@ -86709,7 +86709,7 @@
         </is>
       </c>
       <c r="D4794" t="n">
-        <v>22.6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4795">
@@ -87213,7 +87213,7 @@
         </is>
       </c>
       <c r="D4822" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="4823">
@@ -89931,7 +89931,7 @@
         </is>
       </c>
       <c r="D4973" t="n">
-        <v>10.2</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="4974">
@@ -92200,6 +92200,906 @@
       </c>
       <c r="D5099" t="n">
         <v>3.5</v>
+      </c>
+    </row>
+    <row r="5100">
+      <c r="A5100" t="n">
+        <v>5099</v>
+      </c>
+      <c r="B5100" t="inlineStr">
+        <is>
+          <t>8606110850522</t>
+        </is>
+      </c>
+      <c r="C5100" t="inlineStr">
+        <is>
+          <t>PERFEX COTTON NATURAL 3SL 16/1</t>
+        </is>
+      </c>
+      <c r="D5100" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="5101">
+      <c r="A5101" t="n">
+        <v>5100</v>
+      </c>
+      <c r="B5101" t="inlineStr">
+        <is>
+          <t>8606033742997</t>
+        </is>
+      </c>
+      <c r="C5101" t="inlineStr">
+        <is>
+          <t>CHIPSY REBRASTI CHILI 55G</t>
+        </is>
+      </c>
+      <c r="D5101" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5102">
+      <c r="A5102" t="n">
+        <v>5101</v>
+      </c>
+      <c r="B5102" t="inlineStr">
+        <is>
+          <t>6936756252568</t>
+        </is>
+      </c>
+      <c r="C5102" t="inlineStr">
+        <is>
+          <t>AMOS GUM. BOM. PEELERZ BANANA 65G</t>
+        </is>
+      </c>
+      <c r="D5102" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="5103">
+      <c r="A5103" t="n">
+        <v>5102</v>
+      </c>
+      <c r="B5103" t="inlineStr">
+        <is>
+          <t>6936756288550</t>
+        </is>
+      </c>
+      <c r="C5103" t="inlineStr">
+        <is>
+          <t>AMOS GUM. BOM. PEELERZ BRESKVA 65G</t>
+        </is>
+      </c>
+      <c r="D5103" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="5104">
+      <c r="A5104" t="n">
+        <v>5103</v>
+      </c>
+      <c r="B5104" t="inlineStr">
+        <is>
+          <t>6941308831825</t>
+        </is>
+      </c>
+      <c r="C5104" t="inlineStr">
+        <is>
+          <t>AMOS 4D DINOSAUR GUM. BOM. 72G</t>
+        </is>
+      </c>
+      <c r="D5104" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="5105">
+      <c r="A5105" t="n">
+        <v>5104</v>
+      </c>
+      <c r="B5105" t="inlineStr">
+        <is>
+          <t>4005808135318</t>
+        </is>
+      </c>
+      <c r="C5105" t="inlineStr">
+        <is>
+          <t>NIVEA SAPUN 100G CREME SOFT</t>
+        </is>
+      </c>
+      <c r="D5105" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="5106">
+      <c r="A5106" t="n">
+        <v>5105</v>
+      </c>
+      <c r="B5106" t="inlineStr">
+        <is>
+          <t>4005900217936</t>
+        </is>
+      </c>
+      <c r="C5106" t="inlineStr">
+        <is>
+          <t>NIVEA SAPUN 100G CREME CARE</t>
+        </is>
+      </c>
+      <c r="D5106" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="5107">
+      <c r="A5107" t="n">
+        <v>5106</v>
+      </c>
+      <c r="B5107" t="inlineStr">
+        <is>
+          <t>4012400532629</t>
+        </is>
+      </c>
+      <c r="C5107" t="inlineStr">
+        <is>
+          <t>SAPUN DUG DALLI ZA MRLJE 125G</t>
+        </is>
+      </c>
+      <c r="D5107" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5108">
+      <c r="A5108" t="n">
+        <v>5107</v>
+      </c>
+      <c r="B5108" t="inlineStr">
+        <is>
+          <t>8002910041939</t>
+        </is>
+      </c>
+      <c r="C5108" t="inlineStr">
+        <is>
+          <t>SOLE TVRDI SAPUN BIJELI 2/1</t>
+        </is>
+      </c>
+      <c r="D5108" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="5109">
+      <c r="A5109" t="n">
+        <v>5108</v>
+      </c>
+      <c r="B5109" t="inlineStr">
+        <is>
+          <t>6963656609871</t>
+        </is>
+      </c>
+      <c r="C5109" t="inlineStr">
+        <is>
+          <t>CAPYBARA JAJE SA IGRACKOM</t>
+        </is>
+      </c>
+      <c r="D5109" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5110">
+      <c r="A5110" t="n">
+        <v>5109</v>
+      </c>
+      <c r="B5110" t="inlineStr">
+        <is>
+          <t>6973456871309</t>
+        </is>
+      </c>
+      <c r="C5110" t="inlineStr">
+        <is>
+          <t>CAPYBARA JAJE SA IGRACKOM</t>
+        </is>
+      </c>
+      <c r="D5110" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5111">
+      <c r="A5111" t="n">
+        <v>5110</v>
+      </c>
+      <c r="B5111" t="inlineStr">
+        <is>
+          <t>6932526600010</t>
+        </is>
+      </c>
+      <c r="C5111" t="inlineStr">
+        <is>
+          <t>CAPYBARA SQUISHY IGRACKA</t>
+        </is>
+      </c>
+      <c r="D5111" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5112">
+      <c r="A5112" t="n">
+        <v>5111</v>
+      </c>
+      <c r="B5112" t="inlineStr">
+        <is>
+          <t>0067238891183</t>
+        </is>
+      </c>
+      <c r="C5112" t="inlineStr">
+        <is>
+          <t>DOVE SAPUN 90G BEAUTY CREAM PINK</t>
+        </is>
+      </c>
+      <c r="D5112" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5113">
+      <c r="A5113" t="n">
+        <v>5112</v>
+      </c>
+      <c r="B5113" t="inlineStr">
+        <is>
+          <t>8710447289327</t>
+        </is>
+      </c>
+      <c r="C5113" t="inlineStr">
+        <is>
+          <t>DOVE SAPUN 90G BEAUTY CREAM PINK</t>
+        </is>
+      </c>
+      <c r="D5113" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5114">
+      <c r="A5114" t="n">
+        <v>5113</v>
+      </c>
+      <c r="B5114" t="inlineStr">
+        <is>
+          <t>6973645390475</t>
+        </is>
+      </c>
+      <c r="C5114" t="inlineStr">
+        <is>
+          <t>MARKERI U BOJI 24/1</t>
+        </is>
+      </c>
+      <c r="D5114" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="5115">
+      <c r="A5115" t="n">
+        <v>5114</v>
+      </c>
+      <c r="B5115" t="inlineStr">
+        <is>
+          <t>3875001972918</t>
+        </is>
+      </c>
+      <c r="C5115" t="inlineStr">
+        <is>
+          <t>FLOMASERI 12/1</t>
+        </is>
+      </c>
+      <c r="D5115" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5116">
+      <c r="A5116" t="n">
+        <v>5115</v>
+      </c>
+      <c r="B5116" t="inlineStr">
+        <is>
+          <t>3875001976961</t>
+        </is>
+      </c>
+      <c r="C5116" t="inlineStr">
+        <is>
+          <t>MARKER U BOJI DVOSTRANI 12/1</t>
+        </is>
+      </c>
+      <c r="D5116" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="5117">
+      <c r="A5117" t="n">
+        <v>5116</v>
+      </c>
+      <c r="B5117" t="inlineStr">
+        <is>
+          <t>6941548800568</t>
+        </is>
+      </c>
+      <c r="C5117" t="inlineStr">
+        <is>
+          <t>PEPELJARA KERAMICKA</t>
+        </is>
+      </c>
+      <c r="D5117" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="5118">
+      <c r="A5118" t="n">
+        <v>5117</v>
+      </c>
+      <c r="B5118" t="inlineStr">
+        <is>
+          <t>8056046107137</t>
+        </is>
+      </c>
+      <c r="C5118" t="inlineStr">
+        <is>
+          <t>STAKLENI STALAK</t>
+        </is>
+      </c>
+      <c r="D5118" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="5119">
+      <c r="A5119" t="n">
+        <v>5118</v>
+      </c>
+      <c r="B5119" t="inlineStr">
+        <is>
+          <t>3875001472494</t>
+        </is>
+      </c>
+      <c r="C5119" t="inlineStr">
+        <is>
+          <t>RAM ZA DOKUMENTE A4</t>
+        </is>
+      </c>
+      <c r="D5119" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5120">
+      <c r="A5120" t="n">
+        <v>5119</v>
+      </c>
+      <c r="B5120" t="inlineStr">
+        <is>
+          <t>6985958489241</t>
+        </is>
+      </c>
+      <c r="C5120" t="inlineStr">
+        <is>
+          <t>PAPIRNE KORPICE ZA MAFINE</t>
+        </is>
+      </c>
+      <c r="D5120" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="5121">
+      <c r="A5121" t="n">
+        <v>5120</v>
+      </c>
+      <c r="B5121" t="inlineStr">
+        <is>
+          <t>8956437474650</t>
+        </is>
+      </c>
+      <c r="C5121" t="inlineStr">
+        <is>
+          <t>BOJANKA 26X19CM</t>
+        </is>
+      </c>
+      <c r="D5121" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="5122">
+      <c r="A5122" t="n">
+        <v>5121</v>
+      </c>
+      <c r="B5122" t="inlineStr">
+        <is>
+          <t>3875001470933</t>
+        </is>
+      </c>
+      <c r="C5122" t="inlineStr">
+        <is>
+          <t>BOJANKA SA STIKERIMA</t>
+        </is>
+      </c>
+      <c r="D5122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5123">
+      <c r="A5123" t="n">
+        <v>5122</v>
+      </c>
+      <c r="B5123" t="inlineStr">
+        <is>
+          <t>00005122</t>
+        </is>
+      </c>
+      <c r="C5123" t="inlineStr">
+        <is>
+          <t>JUNECA PLECKA BK</t>
+        </is>
+      </c>
+      <c r="D5123" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5124">
+      <c r="A5124" t="n">
+        <v>5123</v>
+      </c>
+      <c r="B5124" t="inlineStr">
+        <is>
+          <t>3872688008374</t>
+        </is>
+      </c>
+      <c r="C5124" t="inlineStr">
+        <is>
+          <t>VOLIM SECER KOCKA 600G</t>
+        </is>
+      </c>
+      <c r="D5124" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="5125">
+      <c r="A5125" t="n">
+        <v>5124</v>
+      </c>
+      <c r="B5125" t="inlineStr">
+        <is>
+          <t>3859893641008</t>
+        </is>
+      </c>
+      <c r="C5125" t="inlineStr">
+        <is>
+          <t>VIRO BIJELI KRISTAL SECER 1KG</t>
+        </is>
+      </c>
+      <c r="D5125" t="n">
+        <v>1.67</v>
+      </c>
+    </row>
+    <row r="5126">
+      <c r="A5126" t="n">
+        <v>5125</v>
+      </c>
+      <c r="B5126" t="inlineStr">
+        <is>
+          <t>8720181219450</t>
+        </is>
+      </c>
+      <c r="C5126" t="inlineStr">
+        <is>
+          <t>DOVE SAPUN 90G PINK</t>
+        </is>
+      </c>
+      <c r="D5126" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="5127">
+      <c r="A5127" t="n">
+        <v>5126</v>
+      </c>
+      <c r="B5127" t="inlineStr">
+        <is>
+          <t>8720182258397</t>
+        </is>
+      </c>
+      <c r="C5127" t="inlineStr">
+        <is>
+          <t>DOVE NOURISHING OIL&amp;CARE CREAM 90G</t>
+        </is>
+      </c>
+      <c r="D5127" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="5128">
+      <c r="A5128" t="n">
+        <v>5127</v>
+      </c>
+      <c r="B5128" t="inlineStr">
+        <is>
+          <t>3872607000564</t>
+        </is>
+      </c>
+      <c r="C5128" t="inlineStr">
+        <is>
+          <t>TRAVARICA KOSAC 0.10L 37.5% ALK</t>
+        </is>
+      </c>
+      <c r="D5128" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="5129">
+      <c r="A5129" t="n">
+        <v>5128</v>
+      </c>
+      <c r="B5129" t="inlineStr">
+        <is>
+          <t>3871047300739</t>
+        </is>
+      </c>
+      <c r="C5129" t="inlineStr">
+        <is>
+          <t>VRECE ZA ZAMRZIVAC 3KG LD 25/1</t>
+        </is>
+      </c>
+      <c r="D5129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5130">
+      <c r="A5130" t="n">
+        <v>5129</v>
+      </c>
+      <c r="B5130" t="inlineStr">
+        <is>
+          <t>3870081000902</t>
+        </is>
+      </c>
+      <c r="C5130" t="inlineStr">
+        <is>
+          <t>KOLMIX MJES. ZAC. ZA PILET. 125G</t>
+        </is>
+      </c>
+      <c r="D5130" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="5131">
+      <c r="A5131" t="n">
+        <v>5130</v>
+      </c>
+      <c r="B5131" t="inlineStr">
+        <is>
+          <t>3830073000501</t>
+        </is>
+      </c>
+      <c r="C5131" t="inlineStr">
+        <is>
+          <t>IL GATTO CAPITANO PIL. ZA MAC. 80G</t>
+        </is>
+      </c>
+      <c r="D5131" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="5132">
+      <c r="A5132" t="n">
+        <v>5131</v>
+      </c>
+      <c r="B5132" t="inlineStr">
+        <is>
+          <t>3830073000525</t>
+        </is>
+      </c>
+      <c r="C5132" t="inlineStr">
+        <is>
+          <t>IL GATTO CAPITANO ZEC. ZA MAC. 80G</t>
+        </is>
+      </c>
+      <c r="D5132" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="5133">
+      <c r="A5133" t="n">
+        <v>5132</v>
+      </c>
+      <c r="B5133" t="inlineStr">
+        <is>
+          <t>4005808775163</t>
+        </is>
+      </c>
+      <c r="C5133" t="inlineStr">
+        <is>
+          <t>NIVEA KUPKA 250ML MEN FRESH KICK</t>
+        </is>
+      </c>
+      <c r="D5133" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="5134">
+      <c r="A5134" t="n">
+        <v>5133</v>
+      </c>
+      <c r="B5134" t="inlineStr">
+        <is>
+          <t>8410031972719</t>
+        </is>
+      </c>
+      <c r="C5134" t="inlineStr">
+        <is>
+          <t>MINI CHUPA CHUPS LIZALA 120G 20/1</t>
+        </is>
+      </c>
+      <c r="D5134" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="5135">
+      <c r="A5135" t="n">
+        <v>5134</v>
+      </c>
+      <c r="B5135" t="inlineStr">
+        <is>
+          <t>3875001258920</t>
+        </is>
+      </c>
+      <c r="C5135" t="inlineStr">
+        <is>
+          <t>KUHINJSKA KRPA 50X70CM</t>
+        </is>
+      </c>
+      <c r="D5135" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="5136">
+      <c r="A5136" t="n">
+        <v>5135</v>
+      </c>
+      <c r="B5136" t="inlineStr">
+        <is>
+          <t>5903355003847</t>
+        </is>
+      </c>
+      <c r="C5136" t="inlineStr">
+        <is>
+          <t>YORK STIPALJKE 20/1 STANDARD</t>
+        </is>
+      </c>
+      <c r="D5136" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="5137">
+      <c r="A5137" t="n">
+        <v>5136</v>
+      </c>
+      <c r="B5137" t="inlineStr">
+        <is>
+          <t>5903355155348</t>
+        </is>
+      </c>
+      <c r="C5137" t="inlineStr">
+        <is>
+          <t>YORK WC CETKA RESTART</t>
+        </is>
+      </c>
+      <c r="D5137" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="5138">
+      <c r="A5138" t="n">
+        <v>5137</v>
+      </c>
+      <c r="B5138" t="inlineStr">
+        <is>
+          <t>5903355001874</t>
+        </is>
+      </c>
+      <c r="C5138" t="inlineStr">
+        <is>
+          <t>YORK CETVR. KANTA SA CJEDILOM 10L</t>
+        </is>
+      </c>
+      <c r="D5138" t="n">
+        <v>9.300000000000001</v>
+      </c>
+    </row>
+    <row r="5139">
+      <c r="A5139" t="n">
+        <v>5138</v>
+      </c>
+      <c r="B5139" t="inlineStr">
+        <is>
+          <t>8413178402873</t>
+        </is>
+      </c>
+      <c r="C5139" t="inlineStr">
+        <is>
+          <t>VIDAL DVOGLAVI CRVI 90G</t>
+        </is>
+      </c>
+      <c r="D5139" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="5140">
+      <c r="A5140" t="n">
+        <v>5139</v>
+      </c>
+      <c r="B5140" t="inlineStr">
+        <is>
+          <t>8413178402767</t>
+        </is>
+      </c>
+      <c r="C5140" t="inlineStr">
+        <is>
+          <t>VIDAL KORNJACE 90G</t>
+        </is>
+      </c>
+      <c r="D5140" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="5141">
+      <c r="A5141" t="n">
+        <v>5140</v>
+      </c>
+      <c r="B5141" t="inlineStr">
+        <is>
+          <t>8413178391405</t>
+        </is>
+      </c>
+      <c r="C5141" t="inlineStr">
+        <is>
+          <t>VIDAL MARSHMALLOW MIX 50G</t>
+        </is>
+      </c>
+      <c r="D5141" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="5142">
+      <c r="A5142" t="n">
+        <v>5141</v>
+      </c>
+      <c r="B5142" t="inlineStr">
+        <is>
+          <t>8606019650193</t>
+        </is>
+      </c>
+      <c r="C5142" t="inlineStr">
+        <is>
+          <t>NUTRINO LAB FITNESS MIX 180G</t>
+        </is>
+      </c>
+      <c r="D5142" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="5143">
+      <c r="A5143" t="n">
+        <v>5142</v>
+      </c>
+      <c r="B5143" t="inlineStr">
+        <is>
+          <t>3850102018291</t>
+        </is>
+      </c>
+      <c r="C5143" t="inlineStr">
+        <is>
+          <t>DORINA COKOL. RIZA 26G</t>
+        </is>
+      </c>
+      <c r="D5143" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="5144">
+      <c r="A5144" t="n">
+        <v>5143</v>
+      </c>
+      <c r="B5144" t="inlineStr">
+        <is>
+          <t>3850102018642</t>
+        </is>
+      </c>
+      <c r="C5144" t="inlineStr">
+        <is>
+          <t>DORINA COKOL. KREM LJESNIK 37G</t>
+        </is>
+      </c>
+      <c r="D5144" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="5145">
+      <c r="A5145" t="n">
+        <v>5144</v>
+      </c>
+      <c r="B5145" t="inlineStr">
+        <is>
+          <t>3870081000537</t>
+        </is>
+      </c>
+      <c r="C5145" t="inlineStr">
+        <is>
+          <t>KOLMIX DJUMBIR 38G</t>
+        </is>
+      </c>
+      <c r="D5145" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="5146">
+      <c r="A5146" t="n">
+        <v>5145</v>
+      </c>
+      <c r="B5146" t="inlineStr">
+        <is>
+          <t>3870081000605</t>
+        </is>
+      </c>
+      <c r="C5146" t="inlineStr">
+        <is>
+          <t>KOLMIX BIJELI LUK U PRAHU 45G</t>
+        </is>
+      </c>
+      <c r="D5146" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="5147">
+      <c r="A5147" t="n">
+        <v>5146</v>
+      </c>
+      <c r="B5147" t="inlineStr">
+        <is>
+          <t>3831051009134</t>
+        </is>
+      </c>
+      <c r="C5147" t="inlineStr">
+        <is>
+          <t>ZELENE DOLINE JOGURT VAN&amp;JAG 150G</t>
+        </is>
+      </c>
+      <c r="D5147" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="5148">
+      <c r="A5148" t="n">
+        <v>5147</v>
+      </c>
+      <c r="B5148" t="inlineStr">
+        <is>
+          <t>3831051099158</t>
+        </is>
+      </c>
+      <c r="C5148" t="inlineStr">
+        <is>
+          <t>ZELENE DOLINE JOGURT VISNJA 150G</t>
+        </is>
+      </c>
+      <c r="D5148" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="5149">
+      <c r="A5149" t="n">
+        <v>5148</v>
+      </c>
+      <c r="B5149" t="inlineStr">
+        <is>
+          <t>38700132</t>
+        </is>
+      </c>
+      <c r="C5149" t="inlineStr">
+        <is>
+          <t>ARGETA KOKOSIJA PASTETA 45G</t>
+        </is>
+      </c>
+      <c r="D5149" t="n">
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>